<commit_message>
Update roster 10/2026 from web (30 NV)
</commit_message>
<xml_diff>
--- a/data/2026/10.2026/Lịch trực OCD on OCT final 21Sep26.xlsx
+++ b/data/2026/10.2026/Lịch trực OCD on OCT final 21Sep26.xlsx
@@ -3296,16 +3296,16 @@
         <v>Lê Song Huyền Vi</v>
       </c>
       <c r="D34" t="str">
-        <v/>
+        <v>HC</v>
       </c>
       <c r="E34" t="str">
         <v/>
       </c>
       <c r="F34" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="G34" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="H34" t="str">
         <v/>
@@ -3314,7 +3314,7 @@
         <v/>
       </c>
       <c r="J34" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="K34" t="str">
         <v/>
@@ -3326,25 +3326,25 @@
         <v/>
       </c>
       <c r="N34" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="O34" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="P34" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="Q34" t="str">
         <v/>
       </c>
       <c r="R34" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="S34" t="str">
         <v/>
       </c>
       <c r="T34" t="str">
-        <v/>
+        <v>HC</v>
       </c>
       <c r="U34" t="str">
         <v/>
@@ -3389,13 +3389,13 @@
         <v/>
       </c>
       <c r="AI34">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AJ34">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AK34">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AL34">
         <v>0</v>
@@ -3404,7 +3404,7 @@
         <v>0</v>
       </c>
       <c r="AN34">
-        <v>0</v>
+        <v>72</v>
       </c>
     </row>
     <row r="35">
@@ -3418,10 +3418,10 @@
         <v>Đoàn Văn Tây</v>
       </c>
       <c r="D35" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="E35" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="F35" t="str">
         <v/>
@@ -3430,16 +3430,16 @@
         <v/>
       </c>
       <c r="H35" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="I35" t="str">
         <v/>
       </c>
       <c r="J35" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="K35" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="L35" t="str">
         <v/>
@@ -3448,28 +3448,28 @@
         <v/>
       </c>
       <c r="N35" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="O35" t="str">
         <v/>
       </c>
       <c r="P35" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Q35" t="str">
         <v/>
       </c>
       <c r="R35" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="S35" t="str">
         <v/>
       </c>
       <c r="T35" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="U35" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="V35" t="str">
         <v/>
@@ -3514,10 +3514,10 @@
         <v>0</v>
       </c>
       <c r="AJ35">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AK35">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AL35">
         <v>0</v>
@@ -3526,7 +3526,7 @@
         <v>0</v>
       </c>
       <c r="AN35">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="36">
@@ -3540,13 +3540,13 @@
         <v>Nguyễn Thị Mỹ Hương</v>
       </c>
       <c r="D36" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="E36" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="F36" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="G36" t="str">
         <v/>
@@ -3564,34 +3564,34 @@
         <v/>
       </c>
       <c r="L36" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="M36" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="N36" t="str">
-        <v/>
+        <v>HC</v>
       </c>
       <c r="O36" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="P36" t="str">
         <v/>
       </c>
       <c r="Q36" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="R36" t="str">
         <v/>
       </c>
       <c r="S36" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="T36" t="str">
         <v/>
       </c>
       <c r="U36" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="V36" t="str">
         <v/>
@@ -3633,13 +3633,13 @@
         <v/>
       </c>
       <c r="AI36">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ36">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AK36">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AL36">
         <v>0</v>
@@ -3648,7 +3648,7 @@
         <v>0</v>
       </c>
       <c r="AN36">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="37">
@@ -3671,10 +3671,10 @@
         <v/>
       </c>
       <c r="G37" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="H37" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="I37" t="str">
         <v/>
@@ -3683,34 +3683,34 @@
         <v/>
       </c>
       <c r="K37" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="L37" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="M37" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="N37" t="str">
         <v/>
       </c>
       <c r="O37" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="P37" t="str">
         <v/>
       </c>
       <c r="Q37" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="R37" t="str">
         <v/>
       </c>
       <c r="S37" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="T37" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="U37" t="str">
         <v/>
@@ -3758,10 +3758,10 @@
         <v>0</v>
       </c>
       <c r="AJ37">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AK37">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AL37">
         <v>0</v>
@@ -3770,7 +3770,7 @@
         <v>0</v>
       </c>
       <c r="AN37">
-        <v>0</v>
+        <v>72</v>
       </c>
     </row>
     <row r="38">
@@ -3784,55 +3784,55 @@
         <v>Phan Như Ngọc</v>
       </c>
       <c r="D38" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="E38" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="F38" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="G38" t="str">
         <v/>
       </c>
       <c r="H38" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="I38" t="str">
         <v/>
       </c>
       <c r="J38" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="K38" t="str">
         <v/>
       </c>
       <c r="L38" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="M38" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="N38" t="str">
         <v/>
       </c>
       <c r="O38" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="P38" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Q38" t="str">
         <v/>
       </c>
       <c r="R38" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="S38" t="str">
-        <v/>
+        <v>HC</v>
       </c>
       <c r="T38" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="U38" t="str">
         <v/>
@@ -3877,13 +3877,13 @@
         <v/>
       </c>
       <c r="AI38">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ38">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AK38">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AL38">
         <v>0</v>
@@ -3892,7 +3892,7 @@
         <v>0</v>
       </c>
       <c r="AN38">
-        <v>0</v>
+        <v>96</v>
       </c>
     </row>
     <row r="39">
@@ -3906,16 +3906,16 @@
         <v>Phan Hiền Phúc Đạt</v>
       </c>
       <c r="D39" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="E39" t="str">
         <v/>
       </c>
       <c r="F39" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="G39" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="H39" t="str">
         <v/>
@@ -3924,34 +3924,34 @@
         <v/>
       </c>
       <c r="J39" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="K39" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="L39" t="str">
         <v/>
       </c>
       <c r="M39" t="str">
-        <v/>
+        <v>HC</v>
       </c>
       <c r="N39" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="O39" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="P39" t="str">
         <v/>
       </c>
       <c r="Q39" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="R39" t="str">
         <v/>
       </c>
       <c r="S39" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="T39" t="str">
         <v/>
@@ -3999,13 +3999,13 @@
         <v/>
       </c>
       <c r="AI39">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ39">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AK39">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AL39">
         <v>0</v>
@@ -4014,7 +4014,7 @@
         <v>0</v>
       </c>
       <c r="AN39">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="40">
@@ -4031,7 +4031,7 @@
         <v/>
       </c>
       <c r="E40" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="F40" t="str">
         <v/>
@@ -4040,37 +4040,37 @@
         <v/>
       </c>
       <c r="H40" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="I40" t="str">
         <v/>
       </c>
       <c r="J40" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="K40" t="str">
         <v/>
       </c>
       <c r="L40" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="M40" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="N40" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="O40" t="str">
         <v/>
       </c>
       <c r="P40" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Q40" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="R40" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="S40" t="str">
         <v/>
@@ -4124,10 +4124,10 @@
         <v>0</v>
       </c>
       <c r="AJ40">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AK40">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AL40">
         <v>0</v>
@@ -4136,7 +4136,7 @@
         <v>0</v>
       </c>
       <c r="AN40">
-        <v>0</v>
+        <v>72</v>
       </c>
     </row>
     <row r="41">
@@ -4153,16 +4153,16 @@
         <v/>
       </c>
       <c r="E41" t="str">
-        <v/>
+        <v>HC</v>
       </c>
       <c r="F41" t="str">
-        <v/>
+        <v>HC</v>
       </c>
       <c r="G41" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="H41" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="I41" t="str">
         <v/>
@@ -4171,22 +4171,22 @@
         <v/>
       </c>
       <c r="K41" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="L41" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="M41" t="str">
         <v/>
       </c>
       <c r="N41" t="str">
-        <v/>
+        <v>HC</v>
       </c>
       <c r="O41" t="str">
         <v/>
       </c>
       <c r="P41" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="Q41" t="str">
         <v/>
@@ -4195,10 +4195,10 @@
         <v/>
       </c>
       <c r="S41" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="T41" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="U41" t="str">
         <v/>
@@ -4243,13 +4243,13 @@
         <v/>
       </c>
       <c r="AI41">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AJ41">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AK41">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AL41">
         <v>0</v>
@@ -4258,7 +4258,7 @@
         <v>0</v>
       </c>
       <c r="AN41">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update roster 10/2026 from web (34 NV)
</commit_message>
<xml_diff>
--- a/data/2026/10.2026/Lịch trực OCD on OCT final 21Sep26.xlsx
+++ b/data/2026/10.2026/Lịch trực OCD on OCT final 21Sep26.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AM41"/>
+  <dimension ref="A1:AM45"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -687,79 +687,79 @@
         <v/>
       </c>
       <c r="I12" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="J12" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="K12" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="L12" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="M12" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="N12" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="O12" t="str">
         <v>M</v>
       </c>
       <c r="P12" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="Q12" t="str">
         <v>E</v>
       </c>
       <c r="R12" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="S12" t="str">
         <v/>
       </c>
       <c r="T12" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="U12" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="V12" t="str">
         <v>E</v>
       </c>
       <c r="W12" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="X12" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Y12" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="Z12" t="str">
         <v/>
       </c>
       <c r="AA12" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AB12" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AC12" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AD12" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AE12" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AF12" t="str">
-        <v/>
+        <v>NL</v>
       </c>
       <c r="AG12" t="str">
-        <v>NL</v>
+        <v>M</v>
       </c>
       <c r="AH12">
         <v>0</v>
@@ -806,85 +806,85 @@
         <v/>
       </c>
       <c r="I13" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="J13" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="K13" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="L13" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="M13" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="N13" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="O13" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="P13" t="str">
         <v>E</v>
       </c>
       <c r="Q13" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="R13" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="S13" t="str">
         <v>M</v>
       </c>
       <c r="T13" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="U13" t="str">
         <v>E</v>
       </c>
       <c r="V13" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="W13" t="str">
         <v/>
       </c>
       <c r="X13" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Y13" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="Z13" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AA13" t="str">
         <v/>
       </c>
       <c r="AB13" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AC13" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AD13" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AE13" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AF13" t="str">
         <v>M</v>
       </c>
       <c r="AG13" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AH13">
         <v>0</v>
       </c>
       <c r="AI13">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AJ13">
         <v>9</v>
@@ -896,7 +896,7 @@
         <v>0</v>
       </c>
       <c r="AM13">
-        <v>216</v>
+        <v>204</v>
       </c>
     </row>
     <row r="14">
@@ -925,79 +925,79 @@
         <v/>
       </c>
       <c r="I14" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="J14" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="K14" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="L14" t="str">
         <v>E</v>
       </c>
       <c r="M14" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="N14" t="str">
         <v/>
       </c>
       <c r="O14" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="P14" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Q14" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="R14" t="str">
         <v>M</v>
       </c>
       <c r="S14" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="T14" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="U14" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="V14" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="W14" t="str">
         <v/>
       </c>
       <c r="X14" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="Y14" t="str">
         <v>E</v>
       </c>
       <c r="Z14" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AA14" t="str">
         <v/>
       </c>
       <c r="AB14" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AC14" t="str">
         <v>E</v>
       </c>
       <c r="AD14" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AE14" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AF14" t="str">
-        <v>M</v>
+        <v>NL</v>
       </c>
       <c r="AG14" t="str">
-        <v>NL</v>
+        <v>E</v>
       </c>
       <c r="AH14">
         <v>0</v>
@@ -1044,22 +1044,22 @@
         <v>E</v>
       </c>
       <c r="I15" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="J15" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="K15" t="str">
         <v>M</v>
       </c>
       <c r="L15" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="M15" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="N15" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="O15" t="str">
         <v/>
@@ -1071,7 +1071,7 @@
         <v/>
       </c>
       <c r="R15" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="S15" t="str">
         <v>E</v>
@@ -1080,28 +1080,28 @@
         <v>E</v>
       </c>
       <c r="U15" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="V15" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="W15" t="str">
         <v>M</v>
       </c>
       <c r="X15" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="Y15" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Z15" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AA15" t="str">
         <v>M</v>
       </c>
       <c r="AB15" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AC15" t="str">
         <v/>
@@ -1110,7 +1110,7 @@
         <v/>
       </c>
       <c r="AE15" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AF15" t="str">
         <v>E</v>
@@ -1163,16 +1163,16 @@
         <v>M</v>
       </c>
       <c r="I16" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="J16" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="K16" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="L16" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="M16" t="str">
         <v>E</v>
@@ -1181,61 +1181,61 @@
         <v>E</v>
       </c>
       <c r="O16" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="P16" t="str">
         <v/>
       </c>
       <c r="Q16" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="R16" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="S16" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="T16" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="U16" t="str">
         <v/>
       </c>
       <c r="V16" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="W16" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="X16" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Y16" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Z16" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AA16" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AB16" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AC16" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AD16" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AE16" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AF16" t="str">
-        <v>E</v>
+        <v>NL</v>
       </c>
       <c r="AG16" t="str">
-        <v>NL</v>
+        <v/>
       </c>
       <c r="AH16">
         <v>0</v>
@@ -1282,79 +1282,79 @@
         <v>M</v>
       </c>
       <c r="I17" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="J17" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="K17" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="L17" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="M17" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="N17" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="O17" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="P17" t="str">
         <v>M</v>
       </c>
       <c r="Q17" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="R17" t="str">
         <v>E</v>
       </c>
       <c r="S17" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="T17" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="U17" t="str">
         <v>M</v>
       </c>
       <c r="V17" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="W17" t="str">
         <v>E</v>
       </c>
       <c r="X17" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Y17" t="str">
         <v/>
       </c>
       <c r="Z17" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AA17" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AB17" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AC17" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AD17" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AE17" t="str">
         <v/>
       </c>
       <c r="AF17" t="str">
-        <v/>
+        <v>NL</v>
       </c>
       <c r="AG17" t="str">
-        <v>NL</v>
+        <v/>
       </c>
       <c r="AH17">
         <v>0</v>
@@ -1401,10 +1401,10 @@
         <v>E</v>
       </c>
       <c r="I18" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="J18" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="K18" t="str">
         <v>M</v>
@@ -1413,67 +1413,67 @@
         <v>M</v>
       </c>
       <c r="M18" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="N18" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="O18" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="P18" t="str">
         <v>E</v>
       </c>
       <c r="Q18" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="R18" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="S18" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="T18" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="U18" t="str">
         <v/>
       </c>
       <c r="V18" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="W18" t="str">
         <v>M</v>
       </c>
       <c r="X18" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="Y18" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Z18" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AA18" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AB18" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AC18" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AD18" t="str">
         <v/>
       </c>
       <c r="AE18" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AF18" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AG18" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AH18">
         <v>0</v>
@@ -1482,7 +1482,7 @@
         <v>9</v>
       </c>
       <c r="AJ18">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AK18">
         <v>0</v>
@@ -1491,7 +1491,7 @@
         <v>0</v>
       </c>
       <c r="AM18">
-        <v>216</v>
+        <v>204</v>
       </c>
     </row>
     <row r="19">
@@ -1523,76 +1523,76 @@
         <v/>
       </c>
       <c r="J19" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="K19" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="L19" t="str">
         <v/>
       </c>
       <c r="M19" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="N19" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="O19" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="P19" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Q19" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="R19" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="S19" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="T19" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="U19" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="V19" t="str">
-        <v>M</v>
+        <v>P</v>
       </c>
       <c r="W19" t="str">
         <v>P</v>
       </c>
       <c r="X19" t="str">
-        <v>P</v>
+        <v/>
       </c>
       <c r="Y19" t="str">
         <v/>
       </c>
       <c r="Z19" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AA19" t="str">
         <v>E</v>
       </c>
       <c r="AB19" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AC19" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AD19" t="str">
         <v>M</v>
       </c>
       <c r="AE19" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AF19" t="str">
-        <v>E</v>
+        <v>NL</v>
       </c>
       <c r="AG19" t="str">
-        <v>NL</v>
+        <v>SN</v>
       </c>
       <c r="AH19">
         <v>0</v>
@@ -1610,7 +1610,7 @@
         <v>1</v>
       </c>
       <c r="AM19">
-        <v>204</v>
+        <v>212</v>
       </c>
     </row>
     <row r="20">
@@ -1642,25 +1642,25 @@
         <v>M</v>
       </c>
       <c r="J20" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="K20" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="L20" t="str">
         <v>E</v>
       </c>
       <c r="M20" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="N20" t="str">
         <v/>
       </c>
       <c r="O20" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="P20" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="Q20" t="str">
         <v/>
@@ -1669,49 +1669,49 @@
         <v/>
       </c>
       <c r="S20" t="str">
-        <v/>
+        <v>P</v>
       </c>
       <c r="T20" t="str">
+        <v>E</v>
+      </c>
+      <c r="U20" t="str">
+        <v/>
+      </c>
+      <c r="V20" t="str">
+        <v>E</v>
+      </c>
+      <c r="W20" t="str">
+        <v>E</v>
+      </c>
+      <c r="X20" t="str">
+        <v>E</v>
+      </c>
+      <c r="Y20" t="str">
+        <v/>
+      </c>
+      <c r="Z20" t="str">
+        <v>M</v>
+      </c>
+      <c r="AA20" t="str">
+        <v>M</v>
+      </c>
+      <c r="AB20" t="str">
+        <v>M</v>
+      </c>
+      <c r="AC20" t="str">
+        <v/>
+      </c>
+      <c r="AD20" t="str">
+        <v/>
+      </c>
+      <c r="AE20" t="str">
         <v>P</v>
       </c>
-      <c r="U20" t="str">
-        <v>E</v>
-      </c>
-      <c r="V20" t="str">
-        <v/>
-      </c>
-      <c r="W20" t="str">
-        <v>E</v>
-      </c>
-      <c r="X20" t="str">
-        <v>E</v>
-      </c>
-      <c r="Y20" t="str">
-        <v>E</v>
-      </c>
-      <c r="Z20" t="str">
-        <v/>
-      </c>
-      <c r="AA20" t="str">
-        <v>M</v>
-      </c>
-      <c r="AB20" t="str">
-        <v>M</v>
-      </c>
-      <c r="AC20" t="str">
-        <v>M</v>
-      </c>
-      <c r="AD20" t="str">
-        <v/>
-      </c>
-      <c r="AE20" t="str">
-        <v/>
-      </c>
       <c r="AF20" t="str">
-        <v>P</v>
+        <v>NL</v>
       </c>
       <c r="AG20" t="str">
-        <v>NL</v>
+        <v>M</v>
       </c>
       <c r="AH20">
         <v>0</v>
@@ -1758,79 +1758,79 @@
         <v/>
       </c>
       <c r="I21" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="J21" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="K21" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="L21" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="M21" t="str">
         <v/>
       </c>
       <c r="N21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="O21" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="P21" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Q21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="R21" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="S21" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="T21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="U21" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="V21" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="W21" t="str">
         <v/>
       </c>
       <c r="X21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Y21" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="Z21" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AA21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AB21" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AC21" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AD21" t="str">
         <v>E</v>
       </c>
       <c r="AE21" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AF21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AG21" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AH21">
         <v>0</v>
@@ -1839,7 +1839,7 @@
         <v>7</v>
       </c>
       <c r="AJ21">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AK21">
         <v>0</v>
@@ -1848,7 +1848,7 @@
         <v>0</v>
       </c>
       <c r="AM21">
-        <v>204</v>
+        <v>216</v>
       </c>
     </row>
     <row r="22">
@@ -1877,85 +1877,85 @@
         <v/>
       </c>
       <c r="I22" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="J22" t="str">
         <v>E</v>
       </c>
       <c r="K22" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="L22" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="M22" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="N22" t="str">
         <v>E</v>
       </c>
       <c r="O22" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="P22" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Q22" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="R22" t="str">
         <v>E</v>
       </c>
       <c r="S22" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="T22" t="str">
         <v/>
       </c>
       <c r="U22" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="V22" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="W22" t="str">
         <v/>
       </c>
       <c r="X22" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Y22" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="Z22" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AA22" t="str">
         <v/>
       </c>
       <c r="AB22" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AC22" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AD22" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AE22" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AF22" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AG22" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AH22">
         <v>0</v>
       </c>
       <c r="AI22">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AJ22">
         <v>11</v>
@@ -1967,7 +1967,7 @@
         <v>0</v>
       </c>
       <c r="AM22">
-        <v>216</v>
+        <v>204</v>
       </c>
     </row>
     <row r="23">
@@ -1996,64 +1996,64 @@
         <v>E</v>
       </c>
       <c r="I23" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="J23" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="K23" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="L23" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="M23" t="str">
         <v>E</v>
       </c>
       <c r="N23" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="O23" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="P23" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="Q23" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="R23" t="str">
         <v/>
       </c>
       <c r="S23" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="T23" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="U23" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="V23" t="str">
         <v/>
       </c>
       <c r="W23" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="X23" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="Y23" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Z23" t="str">
         <v/>
       </c>
       <c r="AA23" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AB23" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AC23" t="str">
         <v/>
@@ -2062,19 +2062,19 @@
         <v/>
       </c>
       <c r="AE23" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AF23" t="str">
-        <v>E</v>
+        <v>NL</v>
       </c>
       <c r="AG23" t="str">
-        <v>NL</v>
+        <v>M</v>
       </c>
       <c r="AH23">
         <v>0</v>
       </c>
       <c r="AI23">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AJ23">
         <v>7</v>
@@ -2086,7 +2086,7 @@
         <v>1</v>
       </c>
       <c r="AM23">
-        <v>200</v>
+        <v>212</v>
       </c>
     </row>
     <row r="24">
@@ -2115,58 +2115,58 @@
         <v/>
       </c>
       <c r="I24" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="J24" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="K24" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="L24" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="M24" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="N24" t="str">
         <v>M</v>
       </c>
       <c r="O24" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="P24" t="str">
         <v/>
       </c>
       <c r="Q24" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="R24" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="S24" t="str">
         <v/>
       </c>
       <c r="T24" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="U24" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="V24" t="str">
         <v/>
       </c>
       <c r="W24" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="X24" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Y24" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Z24" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AA24" t="str">
         <v>E</v>
@@ -2175,16 +2175,16 @@
         <v>E</v>
       </c>
       <c r="AC24" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AD24" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AE24" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AF24" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AG24" t="str">
         <v>M</v>
@@ -2193,10 +2193,10 @@
         <v>0</v>
       </c>
       <c r="AI24">
+        <v>9</v>
+      </c>
+      <c r="AJ24">
         <v>8</v>
-      </c>
-      <c r="AJ24">
-        <v>9</v>
       </c>
       <c r="AK24">
         <v>0</v>
@@ -2234,79 +2234,79 @@
         <v>E</v>
       </c>
       <c r="I25" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="J25" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="K25" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="L25" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="M25" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="N25" t="str">
         <v/>
       </c>
       <c r="O25" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="P25" t="str">
         <v>E</v>
       </c>
       <c r="Q25" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="R25" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="S25" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="T25" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="U25" t="str">
         <v/>
       </c>
       <c r="V25" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="W25" t="str">
         <v>M</v>
       </c>
       <c r="X25" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="Y25" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Z25" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AA25" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AB25" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AC25" t="str">
         <v>E</v>
       </c>
       <c r="AD25" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AE25" t="str">
         <v/>
       </c>
       <c r="AF25" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AG25" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AH25">
         <v>0</v>
@@ -2315,7 +2315,7 @@
         <v>7</v>
       </c>
       <c r="AJ25">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AK25">
         <v>0</v>
@@ -2324,7 +2324,7 @@
         <v>0</v>
       </c>
       <c r="AM25">
-        <v>204</v>
+        <v>216</v>
       </c>
     </row>
     <row r="26">
@@ -2356,7 +2356,7 @@
         <v>E</v>
       </c>
       <c r="J26" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="K26" t="str">
         <v/>
@@ -2365,67 +2365,67 @@
         <v/>
       </c>
       <c r="M26" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="N26" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="O26" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="P26" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Q26" t="str">
         <v>M</v>
       </c>
       <c r="R26" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="S26" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="T26" t="str">
         <v/>
       </c>
       <c r="U26" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="V26" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="W26" t="str">
         <v>E</v>
       </c>
       <c r="X26" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Y26" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Z26" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AA26" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AB26" t="str">
         <v/>
       </c>
       <c r="AC26" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AD26" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AE26" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AF26" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AG26" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AH26">
         <v>0</v>
@@ -2434,7 +2434,7 @@
         <v>7</v>
       </c>
       <c r="AJ26">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AK26">
         <v>0</v>
@@ -2443,7 +2443,7 @@
         <v>0</v>
       </c>
       <c r="AM26">
-        <v>216</v>
+        <v>204</v>
       </c>
     </row>
     <row r="27">
@@ -2472,76 +2472,76 @@
         <v/>
       </c>
       <c r="I27" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="J27" t="str">
         <v>E</v>
       </c>
       <c r="K27" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="L27" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="M27" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="N27" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="O27" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="P27" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="Q27" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="R27" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="S27" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="T27" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="U27" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="V27" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="W27" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="X27" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="Y27" t="str">
         <v/>
       </c>
       <c r="Z27" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AA27" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AB27" t="str">
         <v/>
       </c>
       <c r="AC27" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AD27" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AE27" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AF27" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AG27" t="str">
         <v>M</v>
@@ -2550,7 +2550,7 @@
         <v>1</v>
       </c>
       <c r="AI27">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AJ27">
         <v>9</v>
@@ -2562,7 +2562,7 @@
         <v>0</v>
       </c>
       <c r="AM27">
-        <v>200</v>
+        <v>212</v>
       </c>
     </row>
     <row r="28">
@@ -2591,79 +2591,79 @@
         <v>E</v>
       </c>
       <c r="I28" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="J28" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="K28" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="L28" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="M28" t="str">
         <v/>
       </c>
       <c r="N28" t="str">
-        <v/>
+        <v>SN</v>
       </c>
       <c r="O28" t="str">
-        <v>SN</v>
+        <v/>
       </c>
       <c r="P28" t="str">
         <v/>
       </c>
       <c r="Q28" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="R28" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="S28" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="T28" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="U28" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="V28" t="str">
         <v/>
       </c>
       <c r="W28" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="X28" t="str">
         <v>E</v>
       </c>
       <c r="Y28" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Z28" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AA28" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AB28" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AC28" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AD28" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AE28" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AF28" t="str">
-        <v>E</v>
+        <v>NL</v>
       </c>
       <c r="AG28" t="str">
-        <v>NL</v>
+        <v/>
       </c>
       <c r="AH28">
         <v>0</v>
@@ -2672,7 +2672,7 @@
         <v>8</v>
       </c>
       <c r="AJ28">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AK28">
         <v>0</v>
@@ -2681,7 +2681,7 @@
         <v>1</v>
       </c>
       <c r="AM28">
-        <v>208</v>
+        <v>196</v>
       </c>
     </row>
     <row r="29">
@@ -2710,7 +2710,7 @@
         <v>M</v>
       </c>
       <c r="I29" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="J29" t="str">
         <v/>
@@ -2722,49 +2722,49 @@
         <v/>
       </c>
       <c r="M29" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="N29" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="O29" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="P29" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Q29" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="R29" t="str">
         <v>E</v>
       </c>
       <c r="S29" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="T29" t="str">
-        <v/>
+        <v>HC</v>
       </c>
       <c r="U29" t="str">
-        <v>HC</v>
+        <v>M</v>
       </c>
       <c r="V29" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="W29" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="X29" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Y29" t="str">
         <v>M</v>
       </c>
       <c r="Z29" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AA29" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AB29" t="str">
         <v>E</v>
@@ -2773,22 +2773,22 @@
         <v>E</v>
       </c>
       <c r="AD29" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AE29" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AF29" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AG29" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AH29">
         <v>1</v>
       </c>
       <c r="AI29">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AJ29">
         <v>9</v>
@@ -2800,7 +2800,7 @@
         <v>0</v>
       </c>
       <c r="AM29">
-        <v>212</v>
+        <v>200</v>
       </c>
     </row>
     <row r="30">
@@ -2829,79 +2829,79 @@
         <v>SN</v>
       </c>
       <c r="I30" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="J30" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="K30" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="L30" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="M30" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="N30" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="O30" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="P30" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Q30" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="R30" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="S30" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="T30" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="U30" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="V30" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="W30" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="X30" t="str">
         <v/>
       </c>
       <c r="Y30" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="Z30" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AA30" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AB30" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AC30" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AD30" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AE30" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AF30" t="str">
-        <v/>
+        <v>NL</v>
       </c>
       <c r="AG30" t="str">
-        <v>NL</v>
+        <v>E</v>
       </c>
       <c r="AH30">
         <v>0</v>
@@ -2910,7 +2910,7 @@
         <v>7</v>
       </c>
       <c r="AJ30">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AK30">
         <v>0</v>
@@ -2919,18 +2919,18 @@
         <v>1</v>
       </c>
       <c r="AM30">
-        <v>196</v>
+        <v>208</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>DSP PQC</v>
+        <v/>
       </c>
       <c r="B31" t="str">
-        <v>41863</v>
+        <v>43311</v>
       </c>
       <c r="C31" t="str">
-        <v>Lê Ngọc Thành Tài</v>
+        <v>Đinh Minh Trí</v>
       </c>
       <c r="D31" t="str">
         <v/>
@@ -2951,76 +2951,76 @@
         <v>E</v>
       </c>
       <c r="J31" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="K31" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="L31" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="M31" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="N31" t="str">
-        <v>M</v>
+        <v>HC</v>
       </c>
       <c r="O31" t="str">
-        <v>HC</v>
+        <v>E</v>
       </c>
       <c r="P31" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Q31" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="R31" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="S31" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="T31" t="str">
         <v/>
       </c>
       <c r="U31" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="V31" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="W31" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="X31" t="str">
         <v/>
       </c>
       <c r="Y31" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Z31" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AA31" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AB31" t="str">
         <v/>
       </c>
       <c r="AC31" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AD31" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AE31" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AF31" t="str">
-        <v>E</v>
+        <v>NL</v>
       </c>
       <c r="AG31" t="str">
-        <v>NL</v>
+        <v/>
       </c>
       <c r="AH31">
         <v>1</v>
@@ -3029,7 +3029,7 @@
         <v>8</v>
       </c>
       <c r="AJ31">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AK31">
         <v>0</v>
@@ -3038,7 +3038,7 @@
         <v>1</v>
       </c>
       <c r="AM31">
-        <v>208</v>
+        <v>196</v>
       </c>
     </row>
     <row r="32">
@@ -3046,10 +3046,10 @@
         <v/>
       </c>
       <c r="B32" t="str">
-        <v>41865</v>
+        <v>43315</v>
       </c>
       <c r="C32" t="str">
-        <v>Nguyễn Đức Lộc</v>
+        <v>Huỳnh Tấn Phước</v>
       </c>
       <c r="D32" t="str">
         <v>M</v>
@@ -3067,79 +3067,79 @@
         <v>E</v>
       </c>
       <c r="I32" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="J32" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="K32" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="L32" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="M32" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="N32" t="str">
         <v>E</v>
       </c>
       <c r="O32" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="P32" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Q32" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="R32" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="S32" t="str">
-        <v/>
+        <v>HC</v>
       </c>
       <c r="T32" t="str">
-        <v>HC</v>
+        <v>M</v>
       </c>
       <c r="U32" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="V32" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="W32" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="X32" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Y32" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="Z32" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AA32" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AB32" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AC32" t="str">
         <v/>
       </c>
       <c r="AD32" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AE32" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AF32" t="str">
         <v>E</v>
       </c>
       <c r="AG32" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AH32">
         <v>1</v>
@@ -3165,10 +3165,10 @@
         <v/>
       </c>
       <c r="B33" t="str">
-        <v>41867</v>
+        <v>43337</v>
       </c>
       <c r="C33" t="str">
-        <v>Phan Thành Nghĩa</v>
+        <v>Vũ Trọng Khánh</v>
       </c>
       <c r="D33" t="str">
         <v/>
@@ -3186,88 +3186,88 @@
         <v/>
       </c>
       <c r="I33" t="str">
-        <v>HC</v>
+        <v/>
       </c>
       <c r="J33" t="str">
         <v/>
       </c>
       <c r="K33" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="L33" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="M33" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="N33" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="O33" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="P33" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="Q33" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="R33" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="S33" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="T33" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="U33" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="V33" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="W33" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="X33" t="str">
         <v>E</v>
       </c>
       <c r="Y33" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Z33" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AA33" t="str">
         <v>M</v>
       </c>
       <c r="AB33" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AC33" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AD33" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AE33" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AF33" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AG33" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AH33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI33">
         <v>7</v>
       </c>
       <c r="AJ33">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AK33">
         <v>0</v>
@@ -3276,18 +3276,18 @@
         <v>0</v>
       </c>
       <c r="AM33">
-        <v>200</v>
+        <v>204</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>BRF SGN</v>
+        <v/>
       </c>
       <c r="B34" t="str">
-        <v>32117</v>
+        <v>43313</v>
       </c>
       <c r="C34" t="str">
-        <v>Lê Song Huyền Vi</v>
+        <v>Cù Trường Phú</v>
       </c>
       <c r="D34" t="str">
         <v>E</v>
@@ -3305,28 +3305,28 @@
         <v/>
       </c>
       <c r="I34" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="J34" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="K34" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="L34" t="str">
         <v>E</v>
       </c>
       <c r="M34" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="N34" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="O34" t="str">
-        <v>M</v>
+        <v>HC</v>
       </c>
       <c r="P34" t="str">
-        <v>HC</v>
+        <v/>
       </c>
       <c r="Q34" t="str">
         <v/>
@@ -3335,22 +3335,22 @@
         <v/>
       </c>
       <c r="S34" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="T34" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="U34" t="str">
         <v>E</v>
       </c>
       <c r="V34" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="W34" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="X34" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="Y34" t="str">
         <v/>
@@ -3362,22 +3362,22 @@
         <v/>
       </c>
       <c r="AB34" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AC34" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AD34" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AE34" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AF34" t="str">
-        <v>M</v>
+        <v>NL</v>
       </c>
       <c r="AG34" t="str">
-        <v>NL</v>
+        <v>M</v>
       </c>
       <c r="AH34">
         <v>1</v>
@@ -3400,13 +3400,13 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v/>
+        <v>DSP PQC</v>
       </c>
       <c r="B35" t="str">
-        <v>32115</v>
+        <v>41863</v>
       </c>
       <c r="C35" t="str">
-        <v>Đoàn Văn Tây</v>
+        <v>Lê Ngọc Thành Tài</v>
       </c>
       <c r="D35" t="str">
         <v/>
@@ -3424,43 +3424,43 @@
         <v/>
       </c>
       <c r="I35" t="str">
-        <v>C9</v>
+        <v/>
       </c>
       <c r="J35" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="K35" t="str">
-        <v>C9</v>
+        <v>E</v>
       </c>
       <c r="L35" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="M35" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="N35" t="str">
-        <v>C9</v>
+        <v>E</v>
       </c>
       <c r="O35" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="P35" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="Q35" t="str">
-        <v>C9</v>
+        <v>E</v>
       </c>
       <c r="R35" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="S35" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="T35" t="str">
-        <v>C9</v>
+        <v>M</v>
       </c>
       <c r="U35" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="V35" t="str">
         <v/>
@@ -3472,31 +3472,31 @@
         <v/>
       </c>
       <c r="Y35" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="Z35" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AA35" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="AB35" t="str">
-        <v>C9</v>
+        <v>E</v>
       </c>
       <c r="AC35" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AD35" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="AE35" t="str">
-        <v>C9</v>
+        <v>E</v>
       </c>
       <c r="AF35" t="str">
-        <v>E</v>
+        <v>NL</v>
       </c>
       <c r="AG35" t="str">
-        <v>NL</v>
+        <v>C9</v>
       </c>
       <c r="AH35">
         <v>0</v>
@@ -3522,10 +3522,10 @@
         <v/>
       </c>
       <c r="B36" t="str">
-        <v>31969</v>
+        <v>41865</v>
       </c>
       <c r="C36" t="str">
-        <v>Nguyễn Thị Mỹ Hương</v>
+        <v>Nguyễn Đức Lộc</v>
       </c>
       <c r="D36" t="str">
         <v>C9</v>
@@ -3546,76 +3546,76 @@
         <v/>
       </c>
       <c r="J36" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="K36" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="L36" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="M36" t="str">
-        <v>C9</v>
+        <v/>
       </c>
       <c r="N36" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="O36" t="str">
         <v>C9</v>
       </c>
       <c r="P36" t="str">
-        <v>C9</v>
+        <v/>
       </c>
       <c r="Q36" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="R36" t="str">
-        <v>C9</v>
+        <v>E</v>
       </c>
       <c r="S36" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="T36" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="U36" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="V36" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="W36" t="str">
-        <v>C9</v>
+        <v/>
       </c>
       <c r="X36" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="Y36" t="str">
-        <v>C9</v>
+        <v/>
       </c>
       <c r="Z36" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="AA36" t="str">
-        <v>C9</v>
+        <v>E</v>
       </c>
       <c r="AB36" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AC36" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="AD36" t="str">
-        <v>C9</v>
+        <v>E</v>
       </c>
       <c r="AE36" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AF36" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="AG36" t="str">
-        <v>C9</v>
+        <v>E</v>
       </c>
       <c r="AH36">
         <v>0</v>
@@ -3624,7 +3624,7 @@
         <v>0</v>
       </c>
       <c r="AJ36">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AK36">
         <v>10</v>
@@ -3633,7 +3633,7 @@
         <v>0</v>
       </c>
       <c r="AM36">
-        <v>204</v>
+        <v>216</v>
       </c>
     </row>
     <row r="37">
@@ -3641,10 +3641,10 @@
         <v/>
       </c>
       <c r="B37" t="str">
-        <v>37388</v>
+        <v>41867</v>
       </c>
       <c r="C37" t="str">
-        <v>Trương Thị Ngọc Loan</v>
+        <v>Phan Thành Nghĩa</v>
       </c>
       <c r="D37" t="str">
         <v/>
@@ -3662,79 +3662,79 @@
         <v>C9</v>
       </c>
       <c r="I37" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="J37" t="str">
-        <v>C9</v>
+        <v/>
       </c>
       <c r="K37" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="L37" t="str">
-        <v>C9</v>
+        <v/>
       </c>
       <c r="M37" t="str">
-        <v/>
+        <v>SN</v>
       </c>
       <c r="N37" t="str">
-        <v>SN</v>
+        <v/>
       </c>
       <c r="O37" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="P37" t="str">
         <v>E</v>
       </c>
       <c r="Q37" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="R37" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="S37" t="str">
-        <v>C9</v>
+        <v>E</v>
       </c>
       <c r="T37" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="U37" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="V37" t="str">
-        <v>C9</v>
+        <v/>
       </c>
       <c r="W37" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="X37" t="str">
-        <v>C9</v>
+        <v/>
       </c>
       <c r="Y37" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="Z37" t="str">
-        <v>C9</v>
+        <v>E</v>
       </c>
       <c r="AA37" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AB37" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="AC37" t="str">
-        <v>C9</v>
+        <v>E</v>
       </c>
       <c r="AD37" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AE37" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="AF37" t="str">
-        <v>C9</v>
+        <v>E</v>
       </c>
       <c r="AG37" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AH37">
         <v>0</v>
@@ -3757,52 +3757,52 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>BRF PQC</v>
+        <v>BRF SGN</v>
       </c>
       <c r="B38" t="str">
-        <v>41366</v>
+        <v>32117</v>
       </c>
       <c r="C38" t="str">
-        <v>Phan Như Ngọc</v>
+        <v>Lê Song Huyền Vi</v>
       </c>
       <c r="D38" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="E38" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="F38" t="str">
         <v/>
       </c>
       <c r="G38" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="H38" t="str">
         <v/>
       </c>
       <c r="I38" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="J38" t="str">
         <v/>
       </c>
       <c r="K38" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="L38" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="M38" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="N38" t="str">
         <v/>
       </c>
       <c r="O38" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="P38" t="str">
-        <v/>
+        <v>HC</v>
       </c>
       <c r="Q38" t="str">
         <v/>
@@ -3814,19 +3814,19 @@
         <v/>
       </c>
       <c r="T38" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="U38" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="V38" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="W38" t="str">
         <v/>
       </c>
       <c r="X38" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Y38" t="str">
         <v/>
@@ -3841,37 +3841,37 @@
         <v/>
       </c>
       <c r="AC38" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AD38" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AE38" t="str">
         <v/>
       </c>
       <c r="AF38" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AG38" t="str">
-        <v/>
+        <v>NL</v>
       </c>
       <c r="AH38">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI38">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AJ38">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AK38">
         <v>0</v>
       </c>
       <c r="AL38">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AM38">
-        <v>0</v>
+        <v>196</v>
       </c>
     </row>
     <row r="39">
@@ -3879,64 +3879,64 @@
         <v/>
       </c>
       <c r="B39" t="str">
-        <v>41861</v>
+        <v>32115</v>
       </c>
       <c r="C39" t="str">
-        <v>Phan Hiền Phúc Đạt</v>
+        <v>Đoàn Văn Tây</v>
       </c>
       <c r="D39" t="str">
         <v/>
       </c>
       <c r="E39" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="F39" t="str">
         <v/>
       </c>
       <c r="G39" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="H39" t="str">
         <v/>
       </c>
       <c r="I39" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="J39" t="str">
         <v/>
       </c>
       <c r="K39" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="L39" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="M39" t="str">
         <v/>
       </c>
       <c r="N39" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="O39" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="P39" t="str">
         <v/>
       </c>
       <c r="Q39" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="R39" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="S39" t="str">
         <v/>
       </c>
       <c r="T39" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="U39" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="V39" t="str">
         <v/>
@@ -3951,46 +3951,46 @@
         <v/>
       </c>
       <c r="Z39" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AA39" t="str">
         <v/>
       </c>
       <c r="AB39" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="AC39" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AD39" t="str">
         <v/>
       </c>
       <c r="AE39" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="AF39" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AG39" t="str">
-        <v/>
+        <v>NL</v>
       </c>
       <c r="AH39">
         <v>0</v>
       </c>
       <c r="AI39">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ39">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AK39">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="AL39">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AM39">
-        <v>0</v>
+        <v>200</v>
       </c>
     </row>
     <row r="40">
@@ -3998,19 +3998,19 @@
         <v/>
       </c>
       <c r="B40" t="str">
-        <v>42791</v>
+        <v>31969</v>
       </c>
       <c r="C40" t="str">
-        <v>Nguyễn Phương Linh</v>
+        <v>Nguyễn Thị Mỹ Hương</v>
       </c>
       <c r="D40" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="E40" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="F40" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="G40" t="str">
         <v/>
@@ -4025,73 +4025,73 @@
         <v/>
       </c>
       <c r="K40" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="L40" t="str">
         <v/>
       </c>
       <c r="M40" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="N40" t="str">
         <v/>
       </c>
       <c r="O40" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="P40" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="Q40" t="str">
         <v/>
       </c>
       <c r="R40" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="S40" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="T40" t="str">
         <v/>
       </c>
       <c r="U40" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="V40" t="str">
         <v/>
       </c>
       <c r="W40" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="X40" t="str">
         <v/>
       </c>
       <c r="Y40" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="Z40" t="str">
         <v/>
       </c>
       <c r="AA40" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="AB40" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AC40" t="str">
         <v/>
       </c>
       <c r="AD40" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="AE40" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AF40" t="str">
         <v/>
       </c>
       <c r="AG40" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="AH40">
         <v>0</v>
@@ -4100,16 +4100,16 @@
         <v>0</v>
       </c>
       <c r="AJ40">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AK40">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="AL40">
         <v>0</v>
       </c>
       <c r="AM40">
-        <v>0</v>
+        <v>204</v>
       </c>
     </row>
     <row r="41">
@@ -4117,123 +4117,599 @@
         <v/>
       </c>
       <c r="B41" t="str">
+        <v>37388</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Trương Thị Ngọc Loan</v>
+      </c>
+      <c r="D41" t="str">
+        <v/>
+      </c>
+      <c r="E41" t="str">
+        <v>M</v>
+      </c>
+      <c r="F41" t="str">
+        <v>C9</v>
+      </c>
+      <c r="G41" t="str">
+        <v/>
+      </c>
+      <c r="H41" t="str">
+        <v>C9</v>
+      </c>
+      <c r="I41" t="str">
+        <v/>
+      </c>
+      <c r="J41" t="str">
+        <v>C9</v>
+      </c>
+      <c r="K41" t="str">
+        <v/>
+      </c>
+      <c r="L41" t="str">
+        <v>C9</v>
+      </c>
+      <c r="M41" t="str">
+        <v/>
+      </c>
+      <c r="N41" t="str">
+        <v>SN</v>
+      </c>
+      <c r="O41" t="str">
+        <v/>
+      </c>
+      <c r="P41" t="str">
+        <v>E</v>
+      </c>
+      <c r="Q41" t="str">
+        <v>E</v>
+      </c>
+      <c r="R41" t="str">
+        <v/>
+      </c>
+      <c r="S41" t="str">
+        <v>C9</v>
+      </c>
+      <c r="T41" t="str">
+        <v>E</v>
+      </c>
+      <c r="U41" t="str">
+        <v/>
+      </c>
+      <c r="V41" t="str">
+        <v>C9</v>
+      </c>
+      <c r="W41" t="str">
+        <v/>
+      </c>
+      <c r="X41" t="str">
+        <v>C9</v>
+      </c>
+      <c r="Y41" t="str">
+        <v/>
+      </c>
+      <c r="Z41" t="str">
+        <v>C9</v>
+      </c>
+      <c r="AA41" t="str">
+        <v>E</v>
+      </c>
+      <c r="AB41" t="str">
+        <v/>
+      </c>
+      <c r="AC41" t="str">
+        <v>C9</v>
+      </c>
+      <c r="AD41" t="str">
+        <v>E</v>
+      </c>
+      <c r="AE41" t="str">
+        <v/>
+      </c>
+      <c r="AF41" t="str">
+        <v>C9</v>
+      </c>
+      <c r="AG41" t="str">
+        <v>E</v>
+      </c>
+      <c r="AH41">
+        <v>0</v>
+      </c>
+      <c r="AI41">
+        <v>1</v>
+      </c>
+      <c r="AJ41">
+        <v>6</v>
+      </c>
+      <c r="AK41">
+        <v>10</v>
+      </c>
+      <c r="AL41">
+        <v>0</v>
+      </c>
+      <c r="AM41">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>BRF PQC</v>
+      </c>
+      <c r="B42" t="str">
+        <v>41366</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Phan Như Ngọc</v>
+      </c>
+      <c r="D42" t="str">
+        <v/>
+      </c>
+      <c r="E42" t="str">
+        <v/>
+      </c>
+      <c r="F42" t="str">
+        <v/>
+      </c>
+      <c r="G42" t="str">
+        <v/>
+      </c>
+      <c r="H42" t="str">
+        <v/>
+      </c>
+      <c r="I42" t="str">
+        <v/>
+      </c>
+      <c r="J42" t="str">
+        <v/>
+      </c>
+      <c r="K42" t="str">
+        <v/>
+      </c>
+      <c r="L42" t="str">
+        <v/>
+      </c>
+      <c r="M42" t="str">
+        <v/>
+      </c>
+      <c r="N42" t="str">
+        <v/>
+      </c>
+      <c r="O42" t="str">
+        <v/>
+      </c>
+      <c r="P42" t="str">
+        <v/>
+      </c>
+      <c r="Q42" t="str">
+        <v/>
+      </c>
+      <c r="R42" t="str">
+        <v/>
+      </c>
+      <c r="S42" t="str">
+        <v/>
+      </c>
+      <c r="T42" t="str">
+        <v/>
+      </c>
+      <c r="U42" t="str">
+        <v/>
+      </c>
+      <c r="V42" t="str">
+        <v/>
+      </c>
+      <c r="W42" t="str">
+        <v/>
+      </c>
+      <c r="X42" t="str">
+        <v/>
+      </c>
+      <c r="Y42" t="str">
+        <v/>
+      </c>
+      <c r="Z42" t="str">
+        <v/>
+      </c>
+      <c r="AA42" t="str">
+        <v/>
+      </c>
+      <c r="AB42" t="str">
+        <v/>
+      </c>
+      <c r="AC42" t="str">
+        <v/>
+      </c>
+      <c r="AD42" t="str">
+        <v/>
+      </c>
+      <c r="AE42" t="str">
+        <v/>
+      </c>
+      <c r="AF42" t="str">
+        <v/>
+      </c>
+      <c r="AG42" t="str">
+        <v/>
+      </c>
+      <c r="AH42">
+        <v>0</v>
+      </c>
+      <c r="AI42">
+        <v>0</v>
+      </c>
+      <c r="AJ42">
+        <v>0</v>
+      </c>
+      <c r="AK42">
+        <v>0</v>
+      </c>
+      <c r="AL42">
+        <v>0</v>
+      </c>
+      <c r="AM42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v/>
+      </c>
+      <c r="B43" t="str">
+        <v>41861</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Phan Hiền Phúc Đạt</v>
+      </c>
+      <c r="D43" t="str">
+        <v/>
+      </c>
+      <c r="E43" t="str">
+        <v/>
+      </c>
+      <c r="F43" t="str">
+        <v/>
+      </c>
+      <c r="G43" t="str">
+        <v/>
+      </c>
+      <c r="H43" t="str">
+        <v/>
+      </c>
+      <c r="I43" t="str">
+        <v/>
+      </c>
+      <c r="J43" t="str">
+        <v/>
+      </c>
+      <c r="K43" t="str">
+        <v/>
+      </c>
+      <c r="L43" t="str">
+        <v/>
+      </c>
+      <c r="M43" t="str">
+        <v/>
+      </c>
+      <c r="N43" t="str">
+        <v/>
+      </c>
+      <c r="O43" t="str">
+        <v/>
+      </c>
+      <c r="P43" t="str">
+        <v/>
+      </c>
+      <c r="Q43" t="str">
+        <v/>
+      </c>
+      <c r="R43" t="str">
+        <v/>
+      </c>
+      <c r="S43" t="str">
+        <v/>
+      </c>
+      <c r="T43" t="str">
+        <v/>
+      </c>
+      <c r="U43" t="str">
+        <v/>
+      </c>
+      <c r="V43" t="str">
+        <v/>
+      </c>
+      <c r="W43" t="str">
+        <v/>
+      </c>
+      <c r="X43" t="str">
+        <v/>
+      </c>
+      <c r="Y43" t="str">
+        <v/>
+      </c>
+      <c r="Z43" t="str">
+        <v/>
+      </c>
+      <c r="AA43" t="str">
+        <v/>
+      </c>
+      <c r="AB43" t="str">
+        <v/>
+      </c>
+      <c r="AC43" t="str">
+        <v/>
+      </c>
+      <c r="AD43" t="str">
+        <v/>
+      </c>
+      <c r="AE43" t="str">
+        <v/>
+      </c>
+      <c r="AF43" t="str">
+        <v/>
+      </c>
+      <c r="AG43" t="str">
+        <v/>
+      </c>
+      <c r="AH43">
+        <v>0</v>
+      </c>
+      <c r="AI43">
+        <v>0</v>
+      </c>
+      <c r="AJ43">
+        <v>0</v>
+      </c>
+      <c r="AK43">
+        <v>0</v>
+      </c>
+      <c r="AL43">
+        <v>0</v>
+      </c>
+      <c r="AM43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v/>
+      </c>
+      <c r="B44" t="str">
+        <v>42791</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Nguyễn Phương Linh</v>
+      </c>
+      <c r="D44" t="str">
+        <v/>
+      </c>
+      <c r="E44" t="str">
+        <v/>
+      </c>
+      <c r="F44" t="str">
+        <v/>
+      </c>
+      <c r="G44" t="str">
+        <v/>
+      </c>
+      <c r="H44" t="str">
+        <v/>
+      </c>
+      <c r="I44" t="str">
+        <v/>
+      </c>
+      <c r="J44" t="str">
+        <v/>
+      </c>
+      <c r="K44" t="str">
+        <v/>
+      </c>
+      <c r="L44" t="str">
+        <v/>
+      </c>
+      <c r="M44" t="str">
+        <v/>
+      </c>
+      <c r="N44" t="str">
+        <v/>
+      </c>
+      <c r="O44" t="str">
+        <v/>
+      </c>
+      <c r="P44" t="str">
+        <v/>
+      </c>
+      <c r="Q44" t="str">
+        <v/>
+      </c>
+      <c r="R44" t="str">
+        <v/>
+      </c>
+      <c r="S44" t="str">
+        <v/>
+      </c>
+      <c r="T44" t="str">
+        <v/>
+      </c>
+      <c r="U44" t="str">
+        <v/>
+      </c>
+      <c r="V44" t="str">
+        <v/>
+      </c>
+      <c r="W44" t="str">
+        <v/>
+      </c>
+      <c r="X44" t="str">
+        <v/>
+      </c>
+      <c r="Y44" t="str">
+        <v/>
+      </c>
+      <c r="Z44" t="str">
+        <v/>
+      </c>
+      <c r="AA44" t="str">
+        <v/>
+      </c>
+      <c r="AB44" t="str">
+        <v/>
+      </c>
+      <c r="AC44" t="str">
+        <v/>
+      </c>
+      <c r="AD44" t="str">
+        <v/>
+      </c>
+      <c r="AE44" t="str">
+        <v/>
+      </c>
+      <c r="AF44" t="str">
+        <v/>
+      </c>
+      <c r="AG44" t="str">
+        <v/>
+      </c>
+      <c r="AH44">
+        <v>0</v>
+      </c>
+      <c r="AI44">
+        <v>0</v>
+      </c>
+      <c r="AJ44">
+        <v>0</v>
+      </c>
+      <c r="AK44">
+        <v>0</v>
+      </c>
+      <c r="AL44">
+        <v>0</v>
+      </c>
+      <c r="AM44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v/>
+      </c>
+      <c r="B45" t="str">
         <v>42789</v>
       </c>
-      <c r="C41" t="str">
+      <c r="C45" t="str">
         <v>Nguyễn Phạm Quỳnh Trang</v>
       </c>
-      <c r="D41" t="str">
-        <v/>
-      </c>
-      <c r="E41" t="str">
-        <v/>
-      </c>
-      <c r="F41" t="str">
-        <v/>
-      </c>
-      <c r="G41" t="str">
-        <v/>
-      </c>
-      <c r="H41" t="str">
-        <v/>
-      </c>
-      <c r="I41" t="str">
-        <v/>
-      </c>
-      <c r="J41" t="str">
-        <v/>
-      </c>
-      <c r="K41" t="str">
-        <v/>
-      </c>
-      <c r="L41" t="str">
-        <v/>
-      </c>
-      <c r="M41" t="str">
-        <v/>
-      </c>
-      <c r="N41" t="str">
-        <v/>
-      </c>
-      <c r="O41" t="str">
-        <v/>
-      </c>
-      <c r="P41" t="str">
-        <v/>
-      </c>
-      <c r="Q41" t="str">
-        <v/>
-      </c>
-      <c r="R41" t="str">
-        <v/>
-      </c>
-      <c r="S41" t="str">
-        <v/>
-      </c>
-      <c r="T41" t="str">
-        <v/>
-      </c>
-      <c r="U41" t="str">
-        <v/>
-      </c>
-      <c r="V41" t="str">
-        <v/>
-      </c>
-      <c r="W41" t="str">
-        <v/>
-      </c>
-      <c r="X41" t="str">
-        <v/>
-      </c>
-      <c r="Y41" t="str">
-        <v/>
-      </c>
-      <c r="Z41" t="str">
-        <v/>
-      </c>
-      <c r="AA41" t="str">
-        <v/>
-      </c>
-      <c r="AB41" t="str">
-        <v/>
-      </c>
-      <c r="AC41" t="str">
-        <v/>
-      </c>
-      <c r="AD41" t="str">
-        <v/>
-      </c>
-      <c r="AE41" t="str">
-        <v/>
-      </c>
-      <c r="AF41" t="str">
-        <v/>
-      </c>
-      <c r="AG41" t="str">
-        <v/>
-      </c>
-      <c r="AH41">
-        <v>0</v>
-      </c>
-      <c r="AI41">
-        <v>0</v>
-      </c>
-      <c r="AJ41">
-        <v>0</v>
-      </c>
-      <c r="AK41">
-        <v>0</v>
-      </c>
-      <c r="AL41">
-        <v>0</v>
-      </c>
-      <c r="AM41">
+      <c r="D45" t="str">
+        <v/>
+      </c>
+      <c r="E45" t="str">
+        <v/>
+      </c>
+      <c r="F45" t="str">
+        <v/>
+      </c>
+      <c r="G45" t="str">
+        <v/>
+      </c>
+      <c r="H45" t="str">
+        <v/>
+      </c>
+      <c r="I45" t="str">
+        <v/>
+      </c>
+      <c r="J45" t="str">
+        <v/>
+      </c>
+      <c r="K45" t="str">
+        <v/>
+      </c>
+      <c r="L45" t="str">
+        <v/>
+      </c>
+      <c r="M45" t="str">
+        <v/>
+      </c>
+      <c r="N45" t="str">
+        <v/>
+      </c>
+      <c r="O45" t="str">
+        <v/>
+      </c>
+      <c r="P45" t="str">
+        <v/>
+      </c>
+      <c r="Q45" t="str">
+        <v/>
+      </c>
+      <c r="R45" t="str">
+        <v/>
+      </c>
+      <c r="S45" t="str">
+        <v/>
+      </c>
+      <c r="T45" t="str">
+        <v/>
+      </c>
+      <c r="U45" t="str">
+        <v/>
+      </c>
+      <c r="V45" t="str">
+        <v/>
+      </c>
+      <c r="W45" t="str">
+        <v/>
+      </c>
+      <c r="X45" t="str">
+        <v/>
+      </c>
+      <c r="Y45" t="str">
+        <v/>
+      </c>
+      <c r="Z45" t="str">
+        <v/>
+      </c>
+      <c r="AA45" t="str">
+        <v/>
+      </c>
+      <c r="AB45" t="str">
+        <v/>
+      </c>
+      <c r="AC45" t="str">
+        <v/>
+      </c>
+      <c r="AD45" t="str">
+        <v/>
+      </c>
+      <c r="AE45" t="str">
+        <v/>
+      </c>
+      <c r="AF45" t="str">
+        <v/>
+      </c>
+      <c r="AG45" t="str">
+        <v/>
+      </c>
+      <c r="AH45">
+        <v>0</v>
+      </c>
+      <c r="AI45">
+        <v>0</v>
+      </c>
+      <c r="AJ45">
+        <v>0</v>
+      </c>
+      <c r="AK45">
+        <v>0</v>
+      </c>
+      <c r="AL45">
+        <v>0</v>
+      </c>
+      <c r="AM45">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AM41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AM45"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>